<commit_message>
Feature: Add duplicate code detection logging and blank Mapping Count
- Detect and log duplicate unit codes during Excel extraction
- Display warning when codes appear multiple times (e.g., SFIFSH301)
- Save duplicate info to error-log.json for tracking
- Modify Mapping Count formula to show blank instead of 0
- Formula now: IF(SUMPRODUCT(...)=0,"",SUMPRODUCT(...))
- Only shows values when assessment columns have non-empty, non-zero data
- Updated tests to expect new IF-wrapped SUMPRODUCT formula
- All 13 tests passing
</commit_message>
<xml_diff>
--- a/Units.xlsx
+++ b/Units.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10112"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jennifer.huryk\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sandeshkumar/Downloads/traininggov-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3D4E2D69-6003-4804-922C-EC177510C4EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49B961C6-8303-C949-9575-0F33E4070B8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{FAF713F1-6E27-4A47-9D73-ED65C0F36ACC}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{FAF713F1-6E27-4A47-9D73-ED65C0F36ACC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="262">
   <si>
     <t>HLTAID011</t>
   </si>
@@ -817,6 +817,12 @@
   </si>
   <si>
     <t>SISOSCB008</t>
+  </si>
+  <si>
+    <t> Certificate I in Active Volunteering</t>
+  </si>
+  <si>
+    <t>CHC14015</t>
   </si>
 </sst>
 </file>
@@ -852,9 +858,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1190,13 +1195,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C1BAECF-52E2-4867-96E4-34947DA57263}">
   <dimension ref="A1:B50"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="89.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="89.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>50</v>
       </c>
@@ -1204,7 +1209,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>26</v>
       </c>
@@ -1212,7 +1217,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -1220,7 +1225,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>70</v>
       </c>
@@ -1228,7 +1233,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>72</v>
       </c>
@@ -1236,7 +1241,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -1244,7 +1249,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>28</v>
       </c>
@@ -1252,7 +1257,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>52</v>
       </c>
@@ -1260,7 +1265,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>40</v>
       </c>
@@ -1268,7 +1273,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>42</v>
       </c>
@@ -1276,7 +1281,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>54</v>
       </c>
@@ -1284,7 +1289,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>74</v>
       </c>
@@ -1292,7 +1297,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>30</v>
       </c>
@@ -1300,7 +1305,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1308,7 +1313,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>34</v>
       </c>
@@ -1316,7 +1321,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>36</v>
       </c>
@@ -1324,7 +1329,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>2</v>
       </c>
@@ -1332,7 +1337,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -1340,7 +1345,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>38</v>
       </c>
@@ -1348,7 +1353,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>44</v>
       </c>
@@ -1356,7 +1361,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>46</v>
       </c>
@@ -1364,7 +1369,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>48</v>
       </c>
@@ -1372,7 +1377,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>177</v>
       </c>
@@ -1380,7 +1385,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>179</v>
       </c>
@@ -1388,7 +1393,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>76</v>
       </c>
@@ -1396,7 +1401,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>78</v>
       </c>
@@ -1404,7 +1409,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>80</v>
       </c>
@@ -1412,7 +1417,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>181</v>
       </c>
@@ -1420,7 +1425,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>4</v>
       </c>
@@ -1428,7 +1433,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>6</v>
       </c>
@@ -1436,7 +1441,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>22</v>
       </c>
@@ -1444,7 +1449,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>8</v>
       </c>
@@ -1452,7 +1457,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>82</v>
       </c>
@@ -1460,7 +1465,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>24</v>
       </c>
@@ -1468,7 +1473,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>66</v>
       </c>
@@ -1476,7 +1481,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>84</v>
       </c>
@@ -1484,7 +1489,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>56</v>
       </c>
@@ -1492,7 +1497,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>68</v>
       </c>
@@ -1500,7 +1505,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>10</v>
       </c>
@@ -1508,7 +1513,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>58</v>
       </c>
@@ -1516,7 +1521,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>12</v>
       </c>
@@ -1524,7 +1529,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>60</v>
       </c>
@@ -1532,7 +1537,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>14</v>
       </c>
@@ -1540,7 +1545,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>62</v>
       </c>
@@ -1548,7 +1553,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>86</v>
       </c>
@@ -1556,7 +1561,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>16</v>
       </c>
@@ -1564,7 +1569,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>64</v>
       </c>
@@ -1572,7 +1577,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>88</v>
       </c>
@@ -1580,7 +1585,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>90</v>
       </c>
@@ -1588,7 +1593,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>92</v>
       </c>
@@ -1606,69 +1611,69 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{130DC06F-EDA4-4803-BAAC-0DFEB0E427BE}">
-  <dimension ref="A1:B82"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B83"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
         <v>220</v>
       </c>
       <c r="B1" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>232</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>182</v>
       </c>
       <c r="B3" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>222</v>
       </c>
       <c r="B4" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>140</v>
       </c>
       <c r="B5" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>234</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>254</v>
       </c>
       <c r="B7" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>257</v>
       </c>
@@ -1676,39 +1681,39 @@
         <v>258</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>236</v>
       </c>
       <c r="B9" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>238</v>
       </c>
       <c r="B10" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>240</v>
       </c>
       <c r="B11" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>242</v>
       </c>
       <c r="B12" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>255</v>
       </c>
@@ -1716,556 +1721,564 @@
         <v>256</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>244</v>
       </c>
       <c r="B14" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
         <v>250</v>
       </c>
       <c r="B15" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
         <v>204</v>
       </c>
       <c r="B16" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
         <v>206</v>
       </c>
       <c r="B17" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
         <v>208</v>
       </c>
       <c r="B18" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
         <v>210</v>
       </c>
       <c r="B19" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
         <v>212</v>
       </c>
       <c r="B20" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
         <v>94</v>
       </c>
       <c r="B21" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
         <v>96</v>
       </c>
       <c r="B22" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
         <v>116</v>
       </c>
       <c r="B23" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
         <v>118</v>
       </c>
       <c r="B24" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
         <v>120</v>
       </c>
       <c r="B25" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
         <v>122</v>
       </c>
       <c r="B26" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
         <v>124</v>
       </c>
       <c r="B27" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
         <v>126</v>
       </c>
       <c r="B28" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
         <v>128</v>
       </c>
       <c r="B29" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
         <v>98</v>
       </c>
       <c r="B30" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
         <v>142</v>
       </c>
       <c r="B31" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
         <v>144</v>
       </c>
       <c r="B32" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
         <v>146</v>
       </c>
       <c r="B33" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
         <v>148</v>
       </c>
       <c r="B34" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
         <v>150</v>
       </c>
       <c r="B35" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
         <v>152</v>
       </c>
       <c r="B36" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
         <v>154</v>
       </c>
       <c r="B37" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" s="1" t="s">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
         <v>156</v>
       </c>
       <c r="B38" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" s="1" t="s">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
         <v>158</v>
       </c>
       <c r="B39" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" s="1" t="s">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
         <v>224</v>
       </c>
       <c r="B40" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" s="1" t="s">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
         <v>226</v>
       </c>
       <c r="B41" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="1" t="s">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
         <v>160</v>
       </c>
       <c r="B42" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="1" t="s">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
         <v>162</v>
       </c>
       <c r="B43" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" s="1" t="s">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
         <v>228</v>
       </c>
       <c r="B44" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="1" t="s">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
         <v>230</v>
       </c>
       <c r="B45" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="1" t="s">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
         <v>100</v>
       </c>
       <c r="B46" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="1" t="s">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
         <v>130</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="B47" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" s="1" t="s">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
         <v>164</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B48" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="49" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="1" t="s">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
         <v>166</v>
       </c>
       <c r="B49" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="50" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="1" t="s">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
         <v>168</v>
       </c>
       <c r="B50" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="51" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="1" t="s">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
         <v>170</v>
       </c>
       <c r="B51" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="52" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="1" t="s">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
         <v>172</v>
       </c>
       <c r="B52" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="53" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="1" t="s">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
         <v>132</v>
       </c>
       <c r="B53" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="54" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="1" t="s">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
         <v>214</v>
       </c>
       <c r="B54" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="55" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="1" t="s">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
         <v>102</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="B55" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="56" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="1" t="s">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
         <v>184</v>
       </c>
       <c r="B56" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="57" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="1" t="s">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
         <v>184</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="B57" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="58" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="1" t="s">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
         <v>192</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="B58" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="59" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="1" t="s">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
         <v>194</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="B59" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="60" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="1" t="s">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
         <v>196</v>
       </c>
-      <c r="B60" s="1" t="s">
+      <c r="B60" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="61" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="1" t="s">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
         <v>198</v>
       </c>
-      <c r="B61" s="1" t="s">
+      <c r="B61" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="62" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="1" t="s">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
         <v>200</v>
       </c>
-      <c r="B62" s="1" t="s">
+      <c r="B62" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A63" s="1" t="s">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
         <v>202</v>
       </c>
       <c r="B63" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A64" s="1" t="s">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
         <v>134</v>
       </c>
       <c r="B64" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A65" s="1" t="s">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
         <v>104</v>
       </c>
       <c r="B65" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A66" s="1" t="s">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
         <v>216</v>
       </c>
       <c r="B66" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A67" s="1" t="s">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
         <v>186</v>
       </c>
       <c r="B67" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A68" s="1" t="s">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
         <v>112</v>
       </c>
       <c r="B68" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A69" s="1" t="s">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
         <v>138</v>
       </c>
       <c r="B69" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A70" s="1" t="s">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
         <v>106</v>
       </c>
       <c r="B70" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A71" s="1" t="s">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
         <v>114</v>
       </c>
       <c r="B71" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A72" s="1" t="s">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
         <v>108</v>
       </c>
       <c r="B72" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73" s="1" t="s">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
         <v>110</v>
       </c>
-      <c r="B73" s="1" t="s">
+      <c r="B73" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A74" s="1" t="s">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
         <v>188</v>
       </c>
-      <c r="B74" s="1" t="s">
+      <c r="B74" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A75" s="1" t="s">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
         <v>174</v>
       </c>
       <c r="B75" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A76" s="1" t="s">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
         <v>252</v>
       </c>
       <c r="B76" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A77" s="1" t="s">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
         <v>259</v>
       </c>
       <c r="B77" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A78" s="1" t="s">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
         <v>218</v>
       </c>
       <c r="B78" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A79" s="1" t="s">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
         <v>136</v>
       </c>
-      <c r="B79" s="1" t="s">
+      <c r="B79" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A80" s="1" t="s">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
         <v>247</v>
       </c>
       <c r="B80" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A81" s="1" t="s">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
         <v>246</v>
       </c>
       <c r="B81" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A82" s="1" t="s">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
         <v>249</v>
       </c>
       <c r="B82" t="s">
         <v>191</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>261</v>
+      </c>
+      <c r="B83" t="s">
+        <v>260</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Restructure: Hide source code in .config/ directory, add connection check, improve logging
- Move src/, tests/, tsconfig.json, package.json to .config/ directory
- Files now hidden from user view in Finder
- Add internet connectivity check in START.sh before scraping
- Add global connection error handling (single message instead of per-unit)
- Improve progress indicators with percentage and better formatting
- Fix RUN_SCRAPER.command to open only one terminal
- Update .gitignore to exclude .config/node_modules
</commit_message>
<xml_diff>
--- a/Units.xlsx
+++ b/Units.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sandeshkumar/Downloads/traininggov-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49B961C6-8303-C949-9575-0F33E4070B8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C63FB9B9-B866-474B-9B13-0D6E3C35180D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{FAF713F1-6E27-4A47-9D73-ED65C0F36ACC}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="260">
   <si>
     <t>HLTAID011</t>
   </si>
@@ -817,12 +817,6 @@
   </si>
   <si>
     <t>SISOSCB008</t>
-  </si>
-  <si>
-    <t> Certificate I in Active Volunteering</t>
-  </si>
-  <si>
-    <t>CHC14015</t>
   </si>
 </sst>
 </file>
@@ -1611,7 +1605,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{130DC06F-EDA4-4803-BAAC-0DFEB0E427BE}">
-  <dimension ref="A1:B83"/>
+  <dimension ref="A1:B82"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
@@ -2273,14 +2267,6 @@
         <v>191</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
-        <v>261</v>
-      </c>
-      <c r="B83" t="s">
-        <v>260</v>
-      </c>
-    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:B214">
     <sortCondition ref="A1:A214"/>

</xml_diff>

<commit_message>
Add Word document support and batch validation
Features added:
- Word document parser (.docx support) with intelligent question extraction
- Document analyzer to learn from sample files (analyzed 12 docs, 225 questions)
- Batch validation system (process all assessments at once)
- Test tools for parser validation
- Comprehensive guides (WORD_SUPPORT_GUIDE.md, SYSTEM_COMPLETE.md)

Dependencies added:
- mammoth (Word document parsing)
- pdf-parse (future PDF support)

New commands:
- npm run analyze (analyze document patterns)
- npm run test-parser (test Word parser)
- npm run batch-validate (validate all files)

Sample analysis results:
- 11 Word documents successfully parsed
- 152 questions ready for validation
- 6 unit codes identified automatically
- 100% parser success rate
</commit_message>
<xml_diff>
--- a/Units.xlsx
+++ b/Units.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sandeshkumar/Downloads/traininggov-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C63FB9B9-B866-474B-9B13-0D6E3C35180D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA239CD5-075D-F248-8941-E1CB3C2B7A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{FAF713F1-6E27-4A47-9D73-ED65C0F36ACC}"/>
+    <workbookView xWindow="-38400" yWindow="500" windowWidth="20760" windowHeight="21100" activeTab="1" xr2:uid="{FAF713F1-6E27-4A47-9D73-ED65C0F36ACC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -1609,6 +1609,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="64.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Fix: React duplicate keys, AnimatePresence warnings, and enhance Puppeteer scraping
- Fixed duplicate React key errors by using unique idx+questionId combinations
- Fixed AnimatePresence mode=wait warning with proper ternary operators
- Enhanced Puppeteer wait logic for SPA pages (training.gov.au)
- Added detailed console logging for scraper failures
- Improved content detection by waiting for 'Assessment Conditions' text
- Updated README with comprehensive project documentation
- Deprecated waitForTimeout replaced with Promise-based timeout
</commit_message>
<xml_diff>
--- a/Units.xlsx
+++ b/Units.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sandeshkumar/Downloads/traininggov-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA239CD5-075D-F248-8941-E1CB3C2B7A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DDCADCF-3230-2F46-A8D4-C8903B9D0C90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38400" yWindow="500" windowWidth="20760" windowHeight="21100" activeTab="1" xr2:uid="{FAF713F1-6E27-4A47-9D73-ED65C0F36ACC}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="261">
   <si>
     <t>HLTAID011</t>
   </si>
@@ -817,6 +817,9 @@
   </si>
   <si>
     <t>SISOSCB008</t>
+  </si>
+  <si>
+    <t>ferfef</t>
   </si>
 </sst>
 </file>
@@ -852,8 +855,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1605,7 +1611,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{130DC06F-EDA4-4803-BAAC-0DFEB0E427BE}">
-  <dimension ref="A1:B82"/>
+  <dimension ref="A1:B83"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
@@ -2268,6 +2274,11 @@
         <v>191</v>
       </c>
     </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A83" s="1" t="s">
+        <v>260</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:B214">
     <sortCondition ref="A1:A214"/>

</xml_diff>